<commit_message>
updated sheet files, added question and solution pattern
</commit_message>
<xml_diff>
--- a/DSA qns info.xlsx
+++ b/DSA qns info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/00cc61b2d0f2ef09/Documents/Anish/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBB3E1B4-ACB8-46AA-A109-0066C2BD7734}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C88EC6B7-C90D-4EEE-9817-5AD4CEDCDE4C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>88. Merge Sorted Array</t>
   </si>
@@ -76,6 +76,27 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>Easy</t>
+  </si>
+  <si>
+    <t>392. Is Subsequence</t>
+  </si>
+  <si>
+    <t>Leetcode</t>
+  </si>
+  <si>
+    <t>Two pointer</t>
+  </si>
+  <si>
+    <t>This is a classic two pointer approach where we loop and and if the s value found in t then  left pointer. Then when the len(s) is equal to left pointer value then s is subsequence of t.</t>
+  </si>
+  <si>
+    <t>When there are two arrays or string  and we need to check values in both arrays then, most of the time we need to loop like the merge array two pointers, then increment the index when we find specific element in an string or array.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/is-subsequence/description/?envType=study-plan-v2&amp;envId=top-interview-150</t>
   </si>
 </sst>
 </file>
@@ -120,10 +141,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -149,6 +169,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,13 +438,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:N9"/>
+  <dimension ref="A4:N10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
     <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="5"/>
-    <col min="7" max="8" width="8.88671875" style="2"/>
+    <col min="6" max="6" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -433,7 +456,7 @@
       <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>9</v>
       </c>
       <c r="I4" t="s">
@@ -447,19 +470,22 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="I8" s="3"/>
+      <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="4" t="s">
         <v>4</v>
       </c>
       <c r="I9" t="s">
@@ -471,14 +497,38 @@
       </c>
       <c r="N9" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A9" r:id="rId1" display="https://leetcode.com/problems/merge-sorted-array/" xr:uid="{E657AFB2-1BE6-4E89-9124-EB9E27F04D80}"/>
     <hyperlink ref="N9" r:id="rId2" xr:uid="{9F29EA48-2482-4273-997C-AB3547674718}"/>
+    <hyperlink ref="N10" r:id="rId3" xr:uid="{7916F796-2302-4786-AB74-260928CDA614}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Leetcode 75. Sort Colors
</commit_message>
<xml_diff>
--- a/DSA qns info.xlsx
+++ b/DSA qns info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/00cc61b2d0f2ef09/Documents/Anish/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C88EC6B7-C90D-4EEE-9817-5AD4CEDCDE4C}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CAB1DBF-80D1-4B25-A85E-0C29ED0B8DCE}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>88. Merge Sorted Array</t>
   </si>
@@ -97,6 +97,24 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/is-subsequence/description/?envType=study-plan-v2&amp;envId=top-interview-150</t>
+  </si>
+  <si>
+    <t>75. Sort Colors</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>We will need total 3 pointers, 1 for tracking 0's, 1 for 2's and 1 for looping the array. If 0 and 2 elements are sorted the 1 automatically gets sorted because its in middle.</t>
+  </si>
+  <si>
+    <t>We will make a while loop, when middle &lt;= right i.e. (traversing pointer &lt; 2's index storing pointer).  When wrote this the loop will only stop if middle pointer index is equal to last element grouping pointer (i.e. right). In this loop we will do swapping based on current element  value as shown in code. Here we will not do swapping when middle == 1 because when 0 and 2 are sorted 1 is automatically sorted as its in middle. We just increment middle by 1.  and element is 2 we swap but do not increment the middle value because middle value is not keeping track of 2.</t>
+  </si>
+  <si>
+    <t>Know, that swapping only happens in 0 and 2 index. Middle is increment in all element except 2 as it's not keeping track of 2.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sort-colors/description/</t>
   </si>
 </sst>
 </file>
@@ -438,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:N10"/>
+  <dimension ref="A4:N11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
@@ -522,13 +540,40 @@
         <v>20</v>
       </c>
     </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" t="s">
+        <v>25</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A9" r:id="rId1" display="https://leetcode.com/problems/merge-sorted-array/" xr:uid="{E657AFB2-1BE6-4E89-9124-EB9E27F04D80}"/>
     <hyperlink ref="N9" r:id="rId2" xr:uid="{9F29EA48-2482-4273-997C-AB3547674718}"/>
     <hyperlink ref="N10" r:id="rId3" xr:uid="{7916F796-2302-4786-AB74-260928CDA614}"/>
+    <hyperlink ref="N11" r:id="rId4" xr:uid="{D2433676-843F-4794-A94C-6F3306B12862}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Brute Force approach for container with most water
</commit_message>
<xml_diff>
--- a/DSA qns info.xlsx
+++ b/DSA qns info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/00cc61b2d0f2ef09/Documents/Anish/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CAB1DBF-80D1-4B25-A85E-0C29ED0B8DCE}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF9BF8C8-1E74-4ECC-A428-954E69D8EADF}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>88. Merge Sorted Array</t>
   </si>
@@ -115,6 +115,21 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/sort-colors/description/</t>
+  </si>
+  <si>
+    <t>11. Container With Most Water</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area = width * minimum height of any one index. You will need bigger width to fill most water. Because the water can spill down you need the wall to be biggest.  The water can be most water only if the minimum height of any two pointer element times the width they cover in those pointer. </t>
+  </si>
+  <si>
+    <t>We know that taking two pointer will be the best approach. We will start left from 0 and right from len(arr) - 1. We initialize an area = []. Here we will store all the area from the two pointers. The formula is width * height of  small wall of any element. after that we will use max_array object that will lookup for maximum value of area arr. To increase and decrease pointers we go with their wall height if left has small than change that pointer in this way we can solve this problem.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/container-with-most-water/description/</t>
+  </si>
+  <si>
+    <t>No, matter how big an element be inside two pointer, if its friend/pointer is small we will go with the small height because the water can only be filled uptill the smallest height practically.  Instead of L * B we should use width * min height of any one element.  The water can cover only till the height of the wall.</t>
   </si>
 </sst>
 </file>
@@ -159,7 +174,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -170,6 +185,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -456,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:N11"/>
+  <dimension ref="A4:N12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
@@ -566,14 +584,42 @@
         <v>26</v>
       </c>
     </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" t="s">
+        <v>29</v>
+      </c>
+      <c r="L12" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A9" r:id="rId1" display="https://leetcode.com/problems/merge-sorted-array/" xr:uid="{E657AFB2-1BE6-4E89-9124-EB9E27F04D80}"/>
     <hyperlink ref="N9" r:id="rId2" xr:uid="{9F29EA48-2482-4273-997C-AB3547674718}"/>
     <hyperlink ref="N10" r:id="rId3" xr:uid="{7916F796-2302-4786-AB74-260928CDA614}"/>
     <hyperlink ref="N11" r:id="rId4" xr:uid="{D2433676-843F-4794-A94C-6F3306B12862}"/>
+    <hyperlink ref="A12" r:id="rId5" display="https://leetcode.com/problems/container-with-most-water/" xr:uid="{CEAD34B3-4825-4244-AAE2-323DF839E921}"/>
+    <hyperlink ref="N12" r:id="rId6" xr:uid="{AF9CEEFC-CD6F-4F59-ADBC-44D84B5F88B0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Optimal solution for Container with most water
</commit_message>
<xml_diff>
--- a/DSA qns info.xlsx
+++ b/DSA qns info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/00cc61b2d0f2ef09/Documents/Anish/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF9BF8C8-1E74-4ECC-A428-954E69D8EADF}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F403796-89AF-4ABF-8C42-93132386E57F}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -123,13 +123,13 @@
     <t xml:space="preserve">Area = width * minimum height of any one index. You will need bigger width to fill most water. Because the water can spill down you need the wall to be biggest.  The water can be most water only if the minimum height of any two pointer element times the width they cover in those pointer. </t>
   </si>
   <si>
-    <t>We know that taking two pointer will be the best approach. We will start left from 0 and right from len(arr) - 1. We initialize an area = []. Here we will store all the area from the two pointers. The formula is width * height of  small wall of any element. after that we will use max_array object that will lookup for maximum value of area arr. To increase and decrease pointers we go with their wall height if left has small than change that pointer in this way we can solve this problem.</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/container-with-most-water/description/</t>
   </si>
   <si>
-    <t>No, matter how big an element be inside two pointer, if its friend/pointer is small we will go with the small height because the water can only be filled uptill the smallest height practically.  Instead of L * B we should use width * min height of any one element.  The water can cover only till the height of the wall.</t>
+    <t>We know that taking two pointer will be the best approach. We will start left from 0 and right from len(arr) - 1. We initialize an area = 0. Here we will store the area from the two pointers. The formula is width * height of  small wall of any element. after that we will use max_array object that will lookup for maximum value of area arr. To increase and decrease pointers we go with their wall height if left has small than change that pointer in this way we can solve this problem. The width of these pointer will be, right - left.</t>
+  </si>
+  <si>
+    <t>No, matter how big an element be inside two pointer, if its friend/pointer is small we will go with the small height because the water can only be filled uptill the smallest height practically.  Instead of L * B we should use width * min height of any one element.  The water can cover only till the height of the wall. and the width will be, right - left.</t>
   </si>
 </sst>
 </file>
@@ -601,13 +601,13 @@
         <v>28</v>
       </c>
       <c r="I12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L12" t="s">
         <v>31</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added notes for 3 sum in excel
</commit_message>
<xml_diff>
--- a/DSA qns info.xlsx
+++ b/DSA qns info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/00cc61b2d0f2ef09/Documents/Anish/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="108" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F403796-89AF-4ABF-8C42-93132386E57F}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="11_F25DC773A252ABDACC1048AF099E69D85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBF6A307-1280-4CAC-87A4-92E9BB9D877E}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>88. Merge Sorted Array</t>
   </si>
@@ -130,6 +130,21 @@
   </si>
   <si>
     <t>No, matter how big an element be inside two pointer, if its friend/pointer is small we will go with the small height because the water can only be filled uptill the smallest height practically.  Instead of L * B we should use width * min height of any one element.  The water can cover only till the height of the wall. and the width will be, right - left.</t>
+  </si>
+  <si>
+    <t>15. 3Sum</t>
+  </si>
+  <si>
+    <t>We need 3 pointer to solve this problem. We also need unique values no repetition. We Sort the array first. Create a loop, then inside it use two pointers (left, right) to find pairs that sum to -element. Skip duplicates to avoid repeating triplets.</t>
+  </si>
+  <si>
+    <t>We first sort the value so that we can use two pointer to find the sum of the three elements. If there is sum equal to 0 then append in result array, and since we donot want a duplicate array check if the current left and left - 1 pointer are same if yes then increment left pointer. And if sum is not 0 then increment or decrement pointers.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/3sum/</t>
+  </si>
+  <si>
+    <t>Move right inward if sum too big, move left inward if sum too small. When sum == 0, record triplet and skip duplicates with the inner while loop. Sorting + duplicate skipping ensures unique triplets. Time complexity: O(n²), Space: O(1) extra.</t>
   </si>
 </sst>
 </file>
@@ -174,7 +189,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -188,6 +203,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -474,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:N12"/>
+  <dimension ref="A4:N13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
@@ -610,6 +628,32 @@
         <v>29</v>
       </c>
     </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" t="s">
+        <v>34</v>
+      </c>
+      <c r="L13" t="s">
+        <v>36</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A9" r:id="rId1" display="https://leetcode.com/problems/merge-sorted-array/" xr:uid="{E657AFB2-1BE6-4E89-9124-EB9E27F04D80}"/>
@@ -618,8 +662,10 @@
     <hyperlink ref="N11" r:id="rId4" xr:uid="{D2433676-843F-4794-A94C-6F3306B12862}"/>
     <hyperlink ref="A12" r:id="rId5" display="https://leetcode.com/problems/container-with-most-water/" xr:uid="{CEAD34B3-4825-4244-AAE2-323DF839E921}"/>
     <hyperlink ref="N12" r:id="rId6" xr:uid="{AF9CEEFC-CD6F-4F59-ADBC-44D84B5F88B0}"/>
+    <hyperlink ref="A13" r:id="rId7" display="https://leetcode.com/problems/3sum/" xr:uid="{7028336F-E778-4D95-9DAE-972AD27C6510}"/>
+    <hyperlink ref="N13" r:id="rId8" xr:uid="{E5BBC79E-36DF-4299-A50D-965FCCE518C5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>